<commit_message>
Updated the scripts and data with the remaining participants
</commit_message>
<xml_diff>
--- a/Data/Participant_info.xlsx
+++ b/Data/Participant_info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Expansion/BME306/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21A6FC26-56D1-A842-A5A6-4276D4A95EA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80937E38-A804-B24D-AF1E-9A1185A0AA6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1080" yWindow="1140" windowWidth="27640" windowHeight="16260" xr2:uid="{745506D4-C856-EA49-8342-C12D376660D2}"/>
   </bookViews>
@@ -719,6 +719,9 @@
       <c r="A19" t="s">
         <v>19</v>
       </c>
+      <c r="B19" s="1">
+        <v>196</v>
+      </c>
       <c r="C19" t="s">
         <v>25</v>
       </c>
@@ -727,6 +730,9 @@
       <c r="A20" t="s">
         <v>20</v>
       </c>
+      <c r="B20" s="1">
+        <v>163</v>
+      </c>
       <c r="C20" t="s">
         <v>24</v>
       </c>
@@ -734,6 +740,9 @@
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>21</v>
+      </c>
+      <c r="B21" s="1">
+        <v>175</v>
       </c>
       <c r="C21" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
The non linearity statistics and prediction plots are all complete
</commit_message>
<xml_diff>
--- a/Data/Participant_info.xlsx
+++ b/Data/Participant_info.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Volumes/Expansion/BME306/Data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80937E38-A804-B24D-AF1E-9A1185A0AA6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF0774CB-E696-054C-9CC8-DFBDEB04553A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1080" yWindow="1140" windowWidth="27640" windowHeight="16260" xr2:uid="{745506D4-C856-EA49-8342-C12D376660D2}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="28">
   <si>
     <t>Sex</t>
   </si>
@@ -120,6 +120,9 @@
   </si>
   <si>
     <t>sample</t>
+  </si>
+  <si>
+    <t>Age</t>
   </si>
 </sst>
 </file>
@@ -505,10 +508,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E6AA0BC-84C6-604F-891D-2323579F11AA}">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="4" max="4" width="13.6640625" customWidth="1"/>
+    <col min="5" max="5" width="34.6640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -519,10 +526,13 @@
         <v>0</v>
       </c>
       <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -532,8 +542,11 @@
       <c r="C2" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D2">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -543,8 +556,11 @@
       <c r="C3" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D3">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -554,8 +570,11 @@
       <c r="C4" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D4">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -565,8 +584,11 @@
       <c r="C5" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D5">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>6</v>
       </c>
@@ -576,8 +598,11 @@
       <c r="C6" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D6">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -587,11 +612,14 @@
       <c r="C7" t="s">
         <v>25</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7">
+        <v>21</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>8</v>
       </c>
@@ -601,8 +629,11 @@
       <c r="C8" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D8">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>9</v>
       </c>
@@ -612,8 +643,11 @@
       <c r="C9" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D9">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>10</v>
       </c>
@@ -623,8 +657,11 @@
       <c r="C10" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D10">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -634,8 +671,11 @@
       <c r="C11" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D11">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -645,8 +685,11 @@
       <c r="C12" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D12">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>13</v>
       </c>
@@ -656,8 +699,11 @@
       <c r="C13" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D13">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>14</v>
       </c>
@@ -667,8 +713,11 @@
       <c r="C14" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D14">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>15</v>
       </c>
@@ -678,8 +727,11 @@
       <c r="C15" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D15">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>16</v>
       </c>
@@ -689,8 +741,11 @@
       <c r="C16" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D16">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>17</v>
       </c>
@@ -700,8 +755,11 @@
       <c r="C17" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D17">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -711,11 +769,14 @@
       <c r="C18" t="s">
         <v>25</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18">
+        <v>24</v>
+      </c>
+      <c r="E18" s="1" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>19</v>
       </c>
@@ -725,8 +786,11 @@
       <c r="C19" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D19">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>20</v>
       </c>
@@ -736,8 +800,11 @@
       <c r="C20" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="D20">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>21</v>
       </c>
@@ -745,6 +812,9 @@
         <v>175</v>
       </c>
       <c r="C21" t="s">
+        <v>24</v>
+      </c>
+      <c r="D21">
         <v>24</v>
       </c>
     </row>

</xml_diff>